<commit_message>
Batch 1: Python chapters 1-4 and LLM chapter 3 from class 01-04 notes; master updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ng7QdNmPkeTth1tmwox3wd
</commit_message>
<xml_diff>
--- a/master/master.xlsx
+++ b/master/master.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3909" uniqueCount="1268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3951" uniqueCount="1300">
   <si>
     <t xml:space="preserve">Master summary (live formulas)</t>
   </si>
@@ -3437,6 +3437,21 @@
     <t xml:space="preserve">classes_summary/01 - 27 Jun - Python Setup &amp; API Basics.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Dev setup with UV and VS Code, Python basics as agent vocabulary, first API call, plain-function tools and a @tool registry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 1 › 1.1 to 1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python book was empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code snippets copied from the summary; tools.py decorator and calculator guard run and checked; currency.py not run (no network)</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC420</t>
   </si>
   <si>
@@ -3446,6 +3461,15 @@
     <t xml:space="preserve">classes_summary/02 - 28 Jun - Python Refresher.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Lists and indexing, classes, dataclasses, decorators, why Python needs Pydantic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 2 › 2.1 to 2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code files _0 to _4 not opened yet (separate rows); dataclass and decorator claims run and checked</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC421</t>
   </si>
   <si>
@@ -3455,6 +3479,15 @@
     <t xml:space="preserve">classes_summary/03 - 4 Jul - Pydantic Deep Dive.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Pydantic BaseModel, Field, validators, nested models, validating LLM JSON; five AI terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 3 › 3.1 to 3.7; LLM › Ch 3 › 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI vocabulary placed in LLM book on your instruction; Pydantic snippets run and checked</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC422</t>
   </si>
   <si>
@@ -3464,6 +3497,15 @@
     <t xml:space="preserve">classes_summary/04 - 5 Jul - Anatomy of an Agent.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Stateless LLM calls, model vs chatbot vs agent, four providers, Pydantic extraction, manual tool call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 4 › 4.1 to 4.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provider code not run (needs API keys); model names may be out of date, flagged in the chapter</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC423</t>
   </si>
   <si>
@@ -3608,6 +3650,21 @@
     <t xml:space="preserve">classes_transcription_summary/01 - 27 June - Python Setup &amp; API Basics.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Class 1 transcript: ground rules, UV room analogy, project mode, VS Code vs Jupyter, API analogy, Q&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 1 › 1.1 to 1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live Q&amp;A table (course fit for non-tech learners, Copilot vs Claude Code, codebase-understanding tools, industry handbook, Copilot Studio); ground rules and job referrals left out as no teaching content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added UV analogy, UV Q&amp;A, why not CMD, VS Code vs Jupyter, timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q&amp;A rows are opinion and logistics; say if you want them in</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC439</t>
   </si>
   <si>
@@ -3617,16 +3674,55 @@
     <t xml:space="preserve">classes_transcription_summary/02 - 28 June - Python Refresher.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Class 2 transcript: Windows fix-up, indexing, BankAccount, dataclasses, decorators, type safety, Pydantic intro, roadmap, Q&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 2 › 2.1 to 2.5; Ch 3 › 3.1, 3.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live Q&amp;A table (framework token cost, GraphQL vs REST, TypeScript for agents, DevOps agents, vibe coding to the Play Store, guardrails, AgentOps timing, 3.0 vs 2.0) and the course roadmap diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added indexing table, self/__init__, gift-wrap analogy, *args/**kwargs, dataclass vs Pydantic table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q&amp;A rows are opinion, scheduling and future topics; say if you want them in</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC440</t>
   </si>
   <si>
     <t xml:space="preserve">classes_transcription_summary/03 - 4 Jul - Pydantic Deep Dive.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Class 3 transcript: why Pydantic, three blueprint styles, optional fields, coercion, Field, special types, validators, nested models, AI vocabulary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 3 › 3.1 to 3.5; LLM › Ch 3 › 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added typing background, comparison table, coercion table, EmailStr/HttpUrl/SecretStr, model_validator and order, inheritance Q&amp;A, AI term analogies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Course news and job reminder left out as no teaching content</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC441</t>
   </si>
   <si>
     <t xml:space="preserve">classes_transcription_summary/04 - 5 Jul - Anatomy of an Agent.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class 4 transcript: stateless calls, context window demo, web app vs API, OpenRouter, brain-memory-tools anatomy, Q&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python › Ch 4 › 4.1, 4.3, 4.7; LLM › Ch 3 › 3.2, 3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added memory and tools build-up, intern analogy, OpenRouter, Q&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recap and song aside left out as no teaching content</t>
   </si>
   <si>
     <t xml:space="preserve">LC442</t>
@@ -4292,15 +4388,15 @@
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A4,Master!$H$2:$H$465,B$3)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A4,Master!$H$2:$H$465,C$3)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A4,Master!$H$2:$H$465,D$3)</f>
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A4,Master!$H$2:$H$465,E$3)</f>
@@ -4466,15 +4562,15 @@
       </c>
       <c r="B10" s="3" t="n">
         <f aca="false">SUM(B4:B9)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C10" s="3" t="n">
         <f aca="false">SUM(C4:C9)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" s="3" t="n">
         <f aca="false">SUM(D4:D9)</f>
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">SUM(E4:E9)</f>
@@ -4531,7 +4627,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">COUNTIF(Master!$K$2:$K$465,A14)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -4545,7 +4641,7 @@
       </c>
       <c r="B15" s="3" t="n">
         <f aca="false">COUNTIF(Master!$K$2:$K$465,A15)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -4573,7 +4669,7 @@
       </c>
       <c r="B17" s="3" t="n">
         <f aca="false">COUNTIF(Master!$K$2:$K$465,A17)</f>
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -4587,7 +4683,7 @@
       </c>
       <c r="B18" s="3" t="n">
         <f aca="false">COUNTIF(Master!$G$2:$G$465,"Read fully")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -4601,7 +4697,7 @@
       </c>
       <c r="B19" s="3" t="n">
         <f aca="false">COUNTIF(Master!$G$2:$G$465,"Not read")</f>
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -18396,25 +18492,35 @@
       <c r="E420" s="3" t="s">
         <v>1136</v>
       </c>
-      <c r="F420" s="3"/>
+      <c r="F420" s="3" t="s">
+        <v>1137</v>
+      </c>
       <c r="G420" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H420" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I420" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I420" s="3" t="s">
+        <v>1138</v>
+      </c>
       <c r="J420" s="3"/>
       <c r="K420" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L420" s="3"/>
-      <c r="M420" s="3"/>
-      <c r="N420" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="L420" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M420" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N420" s="3" t="s">
+        <v>1141</v>
+      </c>
     </row>
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A421" s="3" t="s">
-        <v>1137</v>
+        <v>1142</v>
       </c>
       <c r="B421" s="3" t="s">
         <v>37</v>
@@ -18423,30 +18529,40 @@
         <v>8</v>
       </c>
       <c r="D421" s="3" t="s">
-        <v>1138</v>
+        <v>1143</v>
       </c>
       <c r="E421" s="3" t="s">
-        <v>1139</v>
-      </c>
-      <c r="F421" s="3"/>
+        <v>1144</v>
+      </c>
+      <c r="F421" s="3" t="s">
+        <v>1145</v>
+      </c>
       <c r="G421" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H421" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I421" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I421" s="3" t="s">
+        <v>1146</v>
+      </c>
       <c r="J421" s="3"/>
       <c r="K421" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L421" s="3"/>
-      <c r="M421" s="3"/>
-      <c r="N421" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="L421" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M421" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N421" s="3" t="s">
+        <v>1147</v>
+      </c>
     </row>
     <row r="422" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A422" s="3" t="s">
-        <v>1140</v>
+        <v>1148</v>
       </c>
       <c r="B422" s="3" t="s">
         <v>37</v>
@@ -18455,30 +18571,40 @@
         <v>8</v>
       </c>
       <c r="D422" s="3" t="s">
-        <v>1141</v>
+        <v>1149</v>
       </c>
       <c r="E422" s="3" t="s">
-        <v>1142</v>
-      </c>
-      <c r="F422" s="3"/>
+        <v>1150</v>
+      </c>
+      <c r="F422" s="3" t="s">
+        <v>1151</v>
+      </c>
       <c r="G422" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H422" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I422" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I422" s="3" t="s">
+        <v>1152</v>
+      </c>
       <c r="J422" s="3"/>
       <c r="K422" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L422" s="3"/>
-      <c r="M422" s="3"/>
-      <c r="N422" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="L422" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M422" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N422" s="3" t="s">
+        <v>1153</v>
+      </c>
     </row>
     <row r="423" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A423" s="3" t="s">
-        <v>1143</v>
+        <v>1154</v>
       </c>
       <c r="B423" s="3" t="s">
         <v>37</v>
@@ -18487,30 +18613,40 @@
         <v>8</v>
       </c>
       <c r="D423" s="3" t="s">
-        <v>1144</v>
+        <v>1155</v>
       </c>
       <c r="E423" s="3" t="s">
-        <v>1145</v>
-      </c>
-      <c r="F423" s="3"/>
+        <v>1156</v>
+      </c>
+      <c r="F423" s="3" t="s">
+        <v>1157</v>
+      </c>
       <c r="G423" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H423" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I423" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I423" s="3" t="s">
+        <v>1158</v>
+      </c>
       <c r="J423" s="3"/>
       <c r="K423" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L423" s="3"/>
-      <c r="M423" s="3"/>
-      <c r="N423" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="L423" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M423" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N423" s="3" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A424" s="3" t="s">
-        <v>1146</v>
+        <v>1160</v>
       </c>
       <c r="B424" s="3" t="s">
         <v>37</v>
@@ -18519,10 +18655,10 @@
         <v>9</v>
       </c>
       <c r="D424" s="3" t="s">
-        <v>1147</v>
+        <v>1161</v>
       </c>
       <c r="E424" s="3" t="s">
-        <v>1148</v>
+        <v>1162</v>
       </c>
       <c r="F424" s="3"/>
       <c r="G424" s="3" t="s">
@@ -18542,7 +18678,7 @@
     </row>
     <row r="425" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A425" s="3" t="s">
-        <v>1149</v>
+        <v>1163</v>
       </c>
       <c r="B425" s="3" t="s">
         <v>37</v>
@@ -18551,10 +18687,10 @@
         <v>10</v>
       </c>
       <c r="D425" s="3" t="s">
-        <v>1150</v>
+        <v>1164</v>
       </c>
       <c r="E425" s="3" t="s">
-        <v>1151</v>
+        <v>1165</v>
       </c>
       <c r="F425" s="3"/>
       <c r="G425" s="3" t="s">
@@ -18574,7 +18710,7 @@
     </row>
     <row r="426" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A426" s="3" t="s">
-        <v>1152</v>
+        <v>1166</v>
       </c>
       <c r="B426" s="3" t="s">
         <v>37</v>
@@ -18583,10 +18719,10 @@
         <v>10</v>
       </c>
       <c r="D426" s="3" t="s">
-        <v>1153</v>
+        <v>1167</v>
       </c>
       <c r="E426" s="3" t="s">
-        <v>1154</v>
+        <v>1168</v>
       </c>
       <c r="F426" s="3"/>
       <c r="G426" s="3" t="s">
@@ -18606,7 +18742,7 @@
     </row>
     <row r="427" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A427" s="3" t="s">
-        <v>1155</v>
+        <v>1169</v>
       </c>
       <c r="B427" s="3" t="s">
         <v>37</v>
@@ -18615,10 +18751,10 @@
         <v>9</v>
       </c>
       <c r="D427" s="3" t="s">
-        <v>1156</v>
+        <v>1170</v>
       </c>
       <c r="E427" s="3" t="s">
-        <v>1157</v>
+        <v>1171</v>
       </c>
       <c r="F427" s="3"/>
       <c r="G427" s="3" t="s">
@@ -18638,7 +18774,7 @@
     </row>
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A428" s="3" t="s">
-        <v>1158</v>
+        <v>1172</v>
       </c>
       <c r="B428" s="3" t="s">
         <v>37</v>
@@ -18647,10 +18783,10 @@
         <v>10</v>
       </c>
       <c r="D428" s="3" t="s">
-        <v>1159</v>
+        <v>1173</v>
       </c>
       <c r="E428" s="3" t="s">
-        <v>1160</v>
+        <v>1174</v>
       </c>
       <c r="F428" s="3"/>
       <c r="G428" s="3" t="s">
@@ -18670,7 +18806,7 @@
     </row>
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A429" s="3" t="s">
-        <v>1161</v>
+        <v>1175</v>
       </c>
       <c r="B429" s="3" t="s">
         <v>37</v>
@@ -18679,10 +18815,10 @@
         <v>10</v>
       </c>
       <c r="D429" s="3" t="s">
-        <v>1162</v>
+        <v>1176</v>
       </c>
       <c r="E429" s="3" t="s">
-        <v>1163</v>
+        <v>1177</v>
       </c>
       <c r="F429" s="3"/>
       <c r="G429" s="3" t="s">
@@ -18702,7 +18838,7 @@
     </row>
     <row r="430" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A430" s="3" t="s">
-        <v>1164</v>
+        <v>1178</v>
       </c>
       <c r="B430" s="3" t="s">
         <v>37</v>
@@ -18711,10 +18847,10 @@
         <v>10</v>
       </c>
       <c r="D430" s="3" t="s">
-        <v>1165</v>
+        <v>1179</v>
       </c>
       <c r="E430" s="3" t="s">
-        <v>1166</v>
+        <v>1180</v>
       </c>
       <c r="F430" s="3"/>
       <c r="G430" s="3" t="s">
@@ -18734,7 +18870,7 @@
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A431" s="3" t="s">
-        <v>1167</v>
+        <v>1181</v>
       </c>
       <c r="B431" s="3" t="s">
         <v>37</v>
@@ -18743,10 +18879,10 @@
         <v>10</v>
       </c>
       <c r="D431" s="3" t="s">
-        <v>1168</v>
+        <v>1182</v>
       </c>
       <c r="E431" s="3" t="s">
-        <v>1169</v>
+        <v>1183</v>
       </c>
       <c r="F431" s="3"/>
       <c r="G431" s="3" t="s">
@@ -18766,7 +18902,7 @@
     </row>
     <row r="432" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A432" s="3" t="s">
-        <v>1170</v>
+        <v>1184</v>
       </c>
       <c r="B432" s="3" t="s">
         <v>37</v>
@@ -18775,10 +18911,10 @@
         <v>10</v>
       </c>
       <c r="D432" s="3" t="s">
-        <v>1171</v>
+        <v>1185</v>
       </c>
       <c r="E432" s="3" t="s">
-        <v>1172</v>
+        <v>1186</v>
       </c>
       <c r="F432" s="3"/>
       <c r="G432" s="3" t="s">
@@ -18798,7 +18934,7 @@
     </row>
     <row r="433" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A433" s="3" t="s">
-        <v>1173</v>
+        <v>1187</v>
       </c>
       <c r="B433" s="3" t="s">
         <v>37</v>
@@ -18807,10 +18943,10 @@
         <v>10</v>
       </c>
       <c r="D433" s="3" t="s">
-        <v>1174</v>
+        <v>1188</v>
       </c>
       <c r="E433" s="3" t="s">
-        <v>1175</v>
+        <v>1189</v>
       </c>
       <c r="F433" s="3"/>
       <c r="G433" s="3" t="s">
@@ -18830,7 +18966,7 @@
     </row>
     <row r="434" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="3" t="s">
-        <v>1176</v>
+        <v>1190</v>
       </c>
       <c r="B434" s="3" t="s">
         <v>37</v>
@@ -18839,10 +18975,10 @@
         <v>10</v>
       </c>
       <c r="D434" s="3" t="s">
-        <v>1177</v>
+        <v>1191</v>
       </c>
       <c r="E434" s="3" t="s">
-        <v>1178</v>
+        <v>1192</v>
       </c>
       <c r="F434" s="3"/>
       <c r="G434" s="3" t="s">
@@ -18862,7 +18998,7 @@
     </row>
     <row r="435" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="3" t="s">
-        <v>1179</v>
+        <v>1193</v>
       </c>
       <c r="B435" s="3" t="s">
         <v>37</v>
@@ -18871,10 +19007,10 @@
         <v>11</v>
       </c>
       <c r="D435" s="3" t="s">
-        <v>1180</v>
+        <v>1194</v>
       </c>
       <c r="E435" s="3" t="s">
-        <v>1181</v>
+        <v>1195</v>
       </c>
       <c r="F435" s="3"/>
       <c r="G435" s="3" t="s">
@@ -18894,7 +19030,7 @@
     </row>
     <row r="436" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A436" s="3" t="s">
-        <v>1182</v>
+        <v>1196</v>
       </c>
       <c r="B436" s="3" t="s">
         <v>37</v>
@@ -18903,10 +19039,10 @@
         <v>11</v>
       </c>
       <c r="D436" s="3" t="s">
-        <v>1183</v>
+        <v>1197</v>
       </c>
       <c r="E436" s="3" t="s">
-        <v>1184</v>
+        <v>1198</v>
       </c>
       <c r="F436" s="3"/>
       <c r="G436" s="3" t="s">
@@ -18926,7 +19062,7 @@
     </row>
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A437" s="3" t="s">
-        <v>1185</v>
+        <v>1199</v>
       </c>
       <c r="B437" s="3" t="s">
         <v>37</v>
@@ -18935,10 +19071,10 @@
         <v>11</v>
       </c>
       <c r="D437" s="3" t="s">
-        <v>1186</v>
+        <v>1200</v>
       </c>
       <c r="E437" s="3" t="s">
-        <v>1187</v>
+        <v>1201</v>
       </c>
       <c r="F437" s="3"/>
       <c r="G437" s="3" t="s">
@@ -18958,7 +19094,7 @@
     </row>
     <row r="438" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A438" s="3" t="s">
-        <v>1188</v>
+        <v>1202</v>
       </c>
       <c r="B438" s="3" t="s">
         <v>37</v>
@@ -18967,10 +19103,10 @@
         <v>9</v>
       </c>
       <c r="D438" s="3" t="s">
-        <v>1189</v>
+        <v>1203</v>
       </c>
       <c r="E438" s="3" t="s">
-        <v>1190</v>
+        <v>1204</v>
       </c>
       <c r="F438" s="3"/>
       <c r="G438" s="3" t="s">
@@ -18990,7 +19126,7 @@
     </row>
     <row r="439" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A439" s="3" t="s">
-        <v>1191</v>
+        <v>1205</v>
       </c>
       <c r="B439" s="3" t="s">
         <v>37</v>
@@ -18999,30 +19135,42 @@
         <v>8</v>
       </c>
       <c r="D439" s="3" t="s">
-        <v>1192</v>
+        <v>1206</v>
       </c>
       <c r="E439" s="3" t="s">
-        <v>1193</v>
-      </c>
-      <c r="F439" s="3"/>
+        <v>1207</v>
+      </c>
+      <c r="F439" s="3" t="s">
+        <v>1208</v>
+      </c>
       <c r="G439" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H439" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I439" s="3"/>
-      <c r="J439" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="I439" s="3" t="s">
+        <v>1209</v>
+      </c>
+      <c r="J439" s="3" t="s">
+        <v>1210</v>
+      </c>
       <c r="K439" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L439" s="3"/>
-      <c r="M439" s="3"/>
-      <c r="N439" s="3"/>
+        <v>17</v>
+      </c>
+      <c r="L439" s="3" t="s">
+        <v>1211</v>
+      </c>
+      <c r="M439" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N439" s="3" t="s">
+        <v>1212</v>
+      </c>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A440" s="3" t="s">
-        <v>1194</v>
+        <v>1213</v>
       </c>
       <c r="B440" s="3" t="s">
         <v>37</v>
@@ -19031,30 +19179,42 @@
         <v>8</v>
       </c>
       <c r="D440" s="3" t="s">
-        <v>1195</v>
+        <v>1214</v>
       </c>
       <c r="E440" s="3" t="s">
-        <v>1196</v>
-      </c>
-      <c r="F440" s="3"/>
+        <v>1215</v>
+      </c>
+      <c r="F440" s="3" t="s">
+        <v>1216</v>
+      </c>
       <c r="G440" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H440" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I440" s="3"/>
-      <c r="J440" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="I440" s="3" t="s">
+        <v>1217</v>
+      </c>
+      <c r="J440" s="3" t="s">
+        <v>1218</v>
+      </c>
       <c r="K440" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L440" s="3"/>
-      <c r="M440" s="3"/>
-      <c r="N440" s="3"/>
+        <v>17</v>
+      </c>
+      <c r="L440" s="3" t="s">
+        <v>1219</v>
+      </c>
+      <c r="M440" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N440" s="3" t="s">
+        <v>1220</v>
+      </c>
     </row>
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A441" s="3" t="s">
-        <v>1197</v>
+        <v>1221</v>
       </c>
       <c r="B441" s="3" t="s">
         <v>37</v>
@@ -19063,30 +19223,40 @@
         <v>8</v>
       </c>
       <c r="D441" s="3" t="s">
-        <v>1141</v>
+        <v>1149</v>
       </c>
       <c r="E441" s="3" t="s">
-        <v>1198</v>
-      </c>
-      <c r="F441" s="3"/>
+        <v>1222</v>
+      </c>
+      <c r="F441" s="3" t="s">
+        <v>1223</v>
+      </c>
       <c r="G441" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H441" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I441" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I441" s="3" t="s">
+        <v>1224</v>
+      </c>
       <c r="J441" s="3"/>
       <c r="K441" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L441" s="3"/>
-      <c r="M441" s="3"/>
-      <c r="N441" s="3"/>
+        <v>17</v>
+      </c>
+      <c r="L441" s="3" t="s">
+        <v>1225</v>
+      </c>
+      <c r="M441" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N441" s="3" t="s">
+        <v>1226</v>
+      </c>
     </row>
     <row r="442" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A442" s="3" t="s">
-        <v>1199</v>
+        <v>1227</v>
       </c>
       <c r="B442" s="3" t="s">
         <v>37</v>
@@ -19095,30 +19265,40 @@
         <v>8</v>
       </c>
       <c r="D442" s="3" t="s">
-        <v>1144</v>
+        <v>1155</v>
       </c>
       <c r="E442" s="3" t="s">
-        <v>1200</v>
-      </c>
-      <c r="F442" s="3"/>
+        <v>1228</v>
+      </c>
+      <c r="F442" s="3" t="s">
+        <v>1229</v>
+      </c>
       <c r="G442" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H442" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I442" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I442" s="3" t="s">
+        <v>1230</v>
+      </c>
       <c r="J442" s="3"/>
       <c r="K442" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L442" s="3"/>
-      <c r="M442" s="3"/>
-      <c r="N442" s="3"/>
+        <v>17</v>
+      </c>
+      <c r="L442" s="3" t="s">
+        <v>1231</v>
+      </c>
+      <c r="M442" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N442" s="3" t="s">
+        <v>1232</v>
+      </c>
     </row>
     <row r="443" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A443" s="3" t="s">
-        <v>1201</v>
+        <v>1233</v>
       </c>
       <c r="B443" s="3" t="s">
         <v>37</v>
@@ -19127,10 +19307,10 @@
         <v>9</v>
       </c>
       <c r="D443" s="3" t="s">
-        <v>1202</v>
+        <v>1234</v>
       </c>
       <c r="E443" s="3" t="s">
-        <v>1203</v>
+        <v>1235</v>
       </c>
       <c r="F443" s="3"/>
       <c r="G443" s="3" t="s">
@@ -19150,7 +19330,7 @@
     </row>
     <row r="444" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A444" s="3" t="s">
-        <v>1204</v>
+        <v>1236</v>
       </c>
       <c r="B444" s="3" t="s">
         <v>37</v>
@@ -19159,10 +19339,10 @@
         <v>10</v>
       </c>
       <c r="D444" s="3" t="s">
-        <v>1150</v>
+        <v>1164</v>
       </c>
       <c r="E444" s="3" t="s">
-        <v>1205</v>
+        <v>1237</v>
       </c>
       <c r="F444" s="3"/>
       <c r="G444" s="3" t="s">
@@ -19182,7 +19362,7 @@
     </row>
     <row r="445" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A445" s="3" t="s">
-        <v>1206</v>
+        <v>1238</v>
       </c>
       <c r="B445" s="3" t="s">
         <v>37</v>
@@ -19191,10 +19371,10 @@
         <v>10</v>
       </c>
       <c r="D445" s="3" t="s">
-        <v>1153</v>
+        <v>1167</v>
       </c>
       <c r="E445" s="3" t="s">
-        <v>1207</v>
+        <v>1239</v>
       </c>
       <c r="F445" s="3"/>
       <c r="G445" s="3" t="s">
@@ -19214,7 +19394,7 @@
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A446" s="3" t="s">
-        <v>1208</v>
+        <v>1240</v>
       </c>
       <c r="B446" s="3" t="s">
         <v>37</v>
@@ -19223,10 +19403,10 @@
         <v>9</v>
       </c>
       <c r="D446" s="3" t="s">
-        <v>1209</v>
+        <v>1241</v>
       </c>
       <c r="E446" s="3" t="s">
-        <v>1210</v>
+        <v>1242</v>
       </c>
       <c r="F446" s="3"/>
       <c r="G446" s="3" t="s">
@@ -19246,7 +19426,7 @@
     </row>
     <row r="447" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A447" s="3" t="s">
-        <v>1211</v>
+        <v>1243</v>
       </c>
       <c r="B447" s="3" t="s">
         <v>37</v>
@@ -19255,10 +19435,10 @@
         <v>10</v>
       </c>
       <c r="D447" s="3" t="s">
-        <v>1212</v>
+        <v>1244</v>
       </c>
       <c r="E447" s="3" t="s">
-        <v>1213</v>
+        <v>1245</v>
       </c>
       <c r="F447" s="3"/>
       <c r="G447" s="3" t="s">
@@ -19278,7 +19458,7 @@
     </row>
     <row r="448" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A448" s="3" t="s">
-        <v>1214</v>
+        <v>1246</v>
       </c>
       <c r="B448" s="3" t="s">
         <v>37</v>
@@ -19287,10 +19467,10 @@
         <v>10</v>
       </c>
       <c r="D448" s="3" t="s">
-        <v>1215</v>
+        <v>1247</v>
       </c>
       <c r="E448" s="3" t="s">
-        <v>1216</v>
+        <v>1248</v>
       </c>
       <c r="F448" s="3"/>
       <c r="G448" s="3" t="s">
@@ -19310,7 +19490,7 @@
     </row>
     <row r="449" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A449" s="3" t="s">
-        <v>1217</v>
+        <v>1249</v>
       </c>
       <c r="B449" s="3" t="s">
         <v>37</v>
@@ -19319,10 +19499,10 @@
         <v>10</v>
       </c>
       <c r="D449" s="3" t="s">
-        <v>1218</v>
+        <v>1250</v>
       </c>
       <c r="E449" s="3" t="s">
-        <v>1219</v>
+        <v>1251</v>
       </c>
       <c r="F449" s="3"/>
       <c r="G449" s="3" t="s">
@@ -19342,7 +19522,7 @@
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A450" s="3" t="s">
-        <v>1220</v>
+        <v>1252</v>
       </c>
       <c r="B450" s="3" t="s">
         <v>37</v>
@@ -19351,10 +19531,10 @@
         <v>10</v>
       </c>
       <c r="D450" s="3" t="s">
-        <v>1221</v>
+        <v>1253</v>
       </c>
       <c r="E450" s="3" t="s">
-        <v>1222</v>
+        <v>1254</v>
       </c>
       <c r="F450" s="3"/>
       <c r="G450" s="3" t="s">
@@ -19374,7 +19554,7 @@
     </row>
     <row r="451" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A451" s="3" t="s">
-        <v>1223</v>
+        <v>1255</v>
       </c>
       <c r="B451" s="3" t="s">
         <v>37</v>
@@ -19383,10 +19563,10 @@
         <v>10</v>
       </c>
       <c r="D451" s="3" t="s">
-        <v>1224</v>
+        <v>1256</v>
       </c>
       <c r="E451" s="3" t="s">
-        <v>1225</v>
+        <v>1257</v>
       </c>
       <c r="F451" s="3"/>
       <c r="G451" s="3" t="s">
@@ -19406,7 +19586,7 @@
     </row>
     <row r="452" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A452" s="3" t="s">
-        <v>1226</v>
+        <v>1258</v>
       </c>
       <c r="B452" s="3" t="s">
         <v>37</v>
@@ -19415,10 +19595,10 @@
         <v>10</v>
       </c>
       <c r="D452" s="3" t="s">
-        <v>1227</v>
+        <v>1259</v>
       </c>
       <c r="E452" s="3" t="s">
-        <v>1228</v>
+        <v>1260</v>
       </c>
       <c r="F452" s="3"/>
       <c r="G452" s="3" t="s">
@@ -19438,7 +19618,7 @@
     </row>
     <row r="453" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A453" s="3" t="s">
-        <v>1229</v>
+        <v>1261</v>
       </c>
       <c r="B453" s="3" t="s">
         <v>37</v>
@@ -19447,10 +19627,10 @@
         <v>10</v>
       </c>
       <c r="D453" s="3" t="s">
-        <v>1230</v>
+        <v>1262</v>
       </c>
       <c r="E453" s="3" t="s">
-        <v>1231</v>
+        <v>1263</v>
       </c>
       <c r="F453" s="3"/>
       <c r="G453" s="3" t="s">
@@ -19470,7 +19650,7 @@
     </row>
     <row r="454" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A454" s="3" t="s">
-        <v>1232</v>
+        <v>1264</v>
       </c>
       <c r="B454" s="3" t="s">
         <v>37</v>
@@ -19479,10 +19659,10 @@
         <v>11</v>
       </c>
       <c r="D454" s="3" t="s">
-        <v>1180</v>
+        <v>1194</v>
       </c>
       <c r="E454" s="3" t="s">
-        <v>1233</v>
+        <v>1265</v>
       </c>
       <c r="F454" s="3"/>
       <c r="G454" s="3" t="s">
@@ -19502,7 +19682,7 @@
     </row>
     <row r="455" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A455" s="3" t="s">
-        <v>1234</v>
+        <v>1266</v>
       </c>
       <c r="B455" s="3" t="s">
         <v>37</v>
@@ -19511,10 +19691,10 @@
         <v>11</v>
       </c>
       <c r="D455" s="3" t="s">
-        <v>1235</v>
+        <v>1267</v>
       </c>
       <c r="E455" s="3" t="s">
-        <v>1236</v>
+        <v>1268</v>
       </c>
       <c r="F455" s="3"/>
       <c r="G455" s="3" t="s">
@@ -19534,7 +19714,7 @@
     </row>
     <row r="456" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A456" s="3" t="s">
-        <v>1237</v>
+        <v>1269</v>
       </c>
       <c r="B456" s="3" t="s">
         <v>37</v>
@@ -19543,10 +19723,10 @@
         <v>11</v>
       </c>
       <c r="D456" s="3" t="s">
-        <v>1238</v>
+        <v>1270</v>
       </c>
       <c r="E456" s="3" t="s">
-        <v>1239</v>
+        <v>1271</v>
       </c>
       <c r="F456" s="3"/>
       <c r="G456" s="3" t="s">
@@ -19566,7 +19746,7 @@
     </row>
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A457" s="3" t="s">
-        <v>1240</v>
+        <v>1272</v>
       </c>
       <c r="B457" s="3" t="s">
         <v>37</v>
@@ -19575,10 +19755,10 @@
         <v>11</v>
       </c>
       <c r="D457" s="3" t="s">
-        <v>1241</v>
+        <v>1273</v>
       </c>
       <c r="E457" s="3" t="s">
-        <v>1242</v>
+        <v>1274</v>
       </c>
       <c r="F457" s="3"/>
       <c r="G457" s="3" t="s">
@@ -19598,7 +19778,7 @@
     </row>
     <row r="458" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A458" s="3" t="s">
-        <v>1243</v>
+        <v>1275</v>
       </c>
       <c r="B458" s="3" t="s">
         <v>37</v>
@@ -19607,10 +19787,10 @@
         <v>11</v>
       </c>
       <c r="D458" s="3" t="s">
-        <v>1244</v>
+        <v>1276</v>
       </c>
       <c r="E458" s="3" t="s">
-        <v>1245</v>
+        <v>1277</v>
       </c>
       <c r="F458" s="3"/>
       <c r="G458" s="3" t="s">
@@ -19630,7 +19810,7 @@
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A459" s="3" t="s">
-        <v>1246</v>
+        <v>1278</v>
       </c>
       <c r="B459" s="3" t="s">
         <v>37</v>
@@ -19639,10 +19819,10 @@
         <v>11</v>
       </c>
       <c r="D459" s="3" t="s">
-        <v>1247</v>
+        <v>1279</v>
       </c>
       <c r="E459" s="3" t="s">
-        <v>1248</v>
+        <v>1280</v>
       </c>
       <c r="F459" s="3"/>
       <c r="G459" s="3" t="s">
@@ -19662,7 +19842,7 @@
     </row>
     <row r="460" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A460" s="3" t="s">
-        <v>1249</v>
+        <v>1281</v>
       </c>
       <c r="B460" s="3" t="s">
         <v>37</v>
@@ -19671,10 +19851,10 @@
         <v>11</v>
       </c>
       <c r="D460" s="3" t="s">
-        <v>1250</v>
+        <v>1282</v>
       </c>
       <c r="E460" s="3" t="s">
-        <v>1251</v>
+        <v>1283</v>
       </c>
       <c r="F460" s="3"/>
       <c r="G460" s="3" t="s">
@@ -19694,7 +19874,7 @@
     </row>
     <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A461" s="3" t="s">
-        <v>1252</v>
+        <v>1284</v>
       </c>
       <c r="B461" s="3" t="s">
         <v>37</v>
@@ -19703,10 +19883,10 @@
         <v>10</v>
       </c>
       <c r="D461" s="3" t="s">
-        <v>1253</v>
+        <v>1285</v>
       </c>
       <c r="E461" s="3" t="s">
-        <v>1254</v>
+        <v>1286</v>
       </c>
       <c r="F461" s="3"/>
       <c r="G461" s="3" t="s">
@@ -19726,7 +19906,7 @@
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A462" s="3" t="s">
-        <v>1255</v>
+        <v>1287</v>
       </c>
       <c r="B462" s="3" t="s">
         <v>37</v>
@@ -19735,10 +19915,10 @@
         <v>9</v>
       </c>
       <c r="D462" s="3" t="s">
-        <v>1256</v>
+        <v>1288</v>
       </c>
       <c r="E462" s="3" t="s">
-        <v>1257</v>
+        <v>1289</v>
       </c>
       <c r="F462" s="3"/>
       <c r="G462" s="3" t="s">
@@ -19758,7 +19938,7 @@
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A463" s="3" t="s">
-        <v>1258</v>
+        <v>1290</v>
       </c>
       <c r="B463" s="3" t="s">
         <v>37</v>
@@ -19767,10 +19947,10 @@
         <v>9</v>
       </c>
       <c r="D463" s="3" t="s">
-        <v>1259</v>
+        <v>1291</v>
       </c>
       <c r="E463" s="3" t="s">
-        <v>1260</v>
+        <v>1292</v>
       </c>
       <c r="F463" s="3"/>
       <c r="G463" s="3" t="s">
@@ -19790,7 +19970,7 @@
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A464" s="3" t="s">
-        <v>1261</v>
+        <v>1293</v>
       </c>
       <c r="B464" s="3" t="s">
         <v>37</v>
@@ -19799,10 +19979,10 @@
         <v>11</v>
       </c>
       <c r="D464" s="3" t="s">
-        <v>1262</v>
+        <v>1294</v>
       </c>
       <c r="E464" s="3" t="s">
-        <v>1263</v>
+        <v>1295</v>
       </c>
       <c r="F464" s="3"/>
       <c r="G464" s="3" t="s">
@@ -19822,7 +20002,7 @@
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A465" s="3" t="s">
-        <v>1264</v>
+        <v>1296</v>
       </c>
       <c r="B465" s="3" t="s">
         <v>37</v>
@@ -19831,10 +20011,10 @@
         <v>13</v>
       </c>
       <c r="D465" s="3" t="s">
-        <v>1265</v>
+        <v>1297</v>
       </c>
       <c r="E465" s="3" t="s">
-        <v>1266</v>
+        <v>1298</v>
       </c>
       <c r="F465" s="3"/>
       <c r="G465" s="3" t="s">
@@ -19849,7 +20029,7 @@
         <v>20</v>
       </c>
       <c r="L465" s="3" t="s">
-        <v>1267</v>
+        <v>1299</v>
       </c>
       <c r="M465" s="3"/>
       <c r="N465" s="3"/>

</xml_diff>

<commit_message>
Langchain: split Ch7 into Ch7 (middleware basics) and Ch8 (limits, fallback, PII); later chapters renumbered 9 to 13; master references updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ng7QdLy2CWEArt9UMzAUBr
</commit_message>
<xml_diff>
--- a/master/master.xlsx
+++ b/master/master.xlsx
@@ -2483,10 +2483,10 @@
     <t xml:space="preserve">Whiteboard for classes 11 and 12: hooks loop, HITL intern, summarization 4k trigger, memory before and after, then limits, PII, retries</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 6 › 6.4; Ch 7 › 7.3, 7.5–7.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool selector picture (Drive, Calendar, Gmail, Slack tools), system prompt vs tool description sketch, tool error sketch ('cancel my booking 12345') and the retry delay sketch (4 tries): held for Chapter 8</t>
+    <t xml:space="preserve">Langchain › Ch 6 › 6.4; Ch 7 › 7.3, 7.5, 7.6; Ch 8 › 8.1–8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool selector picture (Drive, Calendar, Gmail, Slack tools), system prompt vs tool description sketch, tool error sketch ('cancel my booking 12345') and the retry delay sketch (4 tries): held for Chapter 9</t>
   </si>
   <si>
     <t xml:space="preserve">Class 11 and 12 halves written. The tool resilience sketches are held for the class 13 batch</t>
@@ -2507,10 +2507,10 @@
     <t xml:space="preserve">Assignment 2 (NovaBank): conceptual and coding questions on agents and prebuilt middleware. Blank question sheet, no answers</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 6 › 6.2, 6.4, 6.9 (A1 Q1 to Q3, B1.1, B1.2); Ch 7 › 7.6 (A2 Q7, B2.1), 7.8 (A2 Q10), 7.10 (B2.2), Practice 11 (B3.1 partly)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1 Q4 (stream_mode), Q5 (name=), A2 Q6, Q8, Q9, A3 Q11 to Q15, B2.3, B3.2, B3.3 and the capstone: they need Chapter 8 and later classes</t>
+    <t xml:space="preserve">Langchain › Ch 6 › 6.2, 6.4, 6.9 (A1 Q1 to Q3, B1.1, B1.2); Ch 7 › 7.6 (A2 Q7, B2.1); Ch 8 › 8.2 (A2 Q10), 8.4 (B2.2), Practice 6 (B3.1 partly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1 Q4 (stream_mode), Q5 (name=), A2 Q6, Q8, Q9, A3 Q11 to Q15, B2.3, B3.2, B3.3 and the capstone: they need Chapter 9 and later classes</t>
   </si>
   <si>
     <t xml:space="preserve">Only the questions the classes so far prepare are listed in Practice. No answers were invented</t>
@@ -2558,10 +2558,10 @@
     <t xml:space="preserve">Read partly</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 7 › 7.4–7.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cells 98 to 101 (to-do list) are read but held for Chapter 8. Cells 102 to 145 are not read yet (class 13: tool selector, tool error, retry, emulator, guardrails)</t>
+    <t xml:space="preserve">Langchain › Ch 7 › 7.4–7.6; Ch 8 › 8.1–8.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cells 98 to 101 (to-do list) are read but held for Chapter 9. Cells 102 to 145 are not read yet (class 13: tool selector, tool error, retry, emulator, guardrails)</t>
   </si>
   <si>
     <t xml:space="preserve">Cells 0 to 97 (class 11 and 12) written. The rest is held for the class 13 batch</t>
@@ -2597,10 +2597,10 @@
     <t xml:space="preserve">Folder README for classes 11 and 12: loop, HITL, summarization, memory, then the nine-middleware table and code</t>
   </si>
   <si>
-    <t xml:space="preserve">Tool error, tool retry formula, tool emulator, to-do list and tool selector entries: held for Chapter 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class 11 and 12 halves written. Five middlewares held for Chapter 8</t>
+    <t xml:space="preserve">Tool error, tool retry formula, tool emulator, to-do list and tool selector entries: held for Chapter 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class 11 and 12 halves written. Five middlewares held for Chapter 9</t>
   </si>
   <si>
     <t xml:space="preserve">LC203</t>
@@ -4568,7 +4568,7 @@
     <t xml:space="preserve">Class 11: agent loop, real tools (TripMate), memory, dynamic tool loading, middleware hooks, summarization, human-in-the-loop, headless tools</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 6 › 6.1–6.8; Ch 7 › 7.1–7.6, 7.13</t>
+    <t xml:space="preserve">Langchain › Ch 6 › 6.1–6.8; Ch 7 › 7.1–7.7</t>
   </si>
   <si>
     <t xml:space="preserve">Chapters 6 and 7 were empty</t>
@@ -4589,13 +4589,13 @@
     <t xml:space="preserve">Class 12 summary: nine built-in middlewares with code (call limits, fallback, PII, to-do list, tool selector, tool error, tool retry, tool emulator), guardrail vs middleware, real-world mapping</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 7 › 7.5, 7.7–7.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To-do list, LLM tool selector, tool error, tool retry and tool emulator sections: held for Chapter 8 together with class 13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Six middlewares and the guardrail idea written. The other five belong with Chapter 8 (to-do lists and tool resilience)</t>
+    <t xml:space="preserve">Langchain › Ch 7 › 7.5; Ch 8 › 8.1–8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To-do list, LLM tool selector, tool error, tool retry and tool emulator sections: held for Chapter 9 together with class 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Six middlewares and the guardrail idea written. The other five belong with Chapter 9 (to-do lists and tool resilience)</t>
   </si>
   <si>
     <t xml:space="preserve">Checked offline: the summary says the card number was masked but the notebook output shows it was not (checksum); the compiled-regex detector raises TypeError</t>
@@ -4907,7 +4907,7 @@
     <t xml:space="preserve">Class 12 transcript summary: why middleware, summarization, HITL, model and tool call limits, model fallback, PII, several middlewares, LangChain vs LangGraph, Q&amp;A</t>
   </si>
   <si>
-    <t xml:space="preserve">Langchain › Ch 7 › 7.3, 7.5, 7.6, 7.7–7.13</t>
+    <t xml:space="preserve">Langchain › Ch 7 › 7.3, 7.5, 7.6; Ch 8 › 8.1–8.7</t>
   </si>
   <si>
     <t xml:space="preserve">Chapter 7 had only the class 11 part</t>

</xml_diff>

<commit_message>
MCP book: Chapters 7-8 (class 22, interview questions); master updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ng7QdLy2CWEArt9UMzAUBr
</commit_message>
<xml_diff>
--- a/master/master.xlsx
+++ b/master/master.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4736" uniqueCount="1829">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4742" uniqueCount="1835">
   <si>
     <t xml:space="preserve">Master summary (live formulas)</t>
   </si>
@@ -5439,6 +5439,15 @@
     <t xml:space="preserve">classes_transcription_summary/22 - 20 Sep - Legacy vs Modern MCP.md</t>
   </si>
   <si>
+    <t xml:space="preserve">MCP › Ch7 Legacy vs modern MCP (7.1-7.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modern requests over HTTP, MRTR elicitation, a full sampling run and progress reporting were not run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class 22 (20 Sep): timeline, stateless idea, removed vs deprecated, client modes, sampling, elicitation, ping, timeouts, LangChain link. Run and checked on fastmcp 4.1.4 and against the official changelog</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC460</t>
   </si>
   <si>
@@ -5500,6 +5509,15 @@
   </si>
   <si>
     <t xml:space="preserve">interview-questions/mcp.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP › Ch8 Interview questions (8.1-8.9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OAuth, scopes and gateway answers are from the file only, not run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Course interview file: 8 production questions. Replica, idempotency, error and spec claims tested; three corrections shown (stateless flag on constructor, bad parameters as isError results, list_changed not sent in test)</t>
   </si>
   <si>
     <t xml:space="preserve">LC464</t>
@@ -5697,11 +5715,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5709,23 +5727,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6194,7 +6212,7 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A8,Master!$H$2:$H$465,B$3)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C8" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A8,Master!$H$2:$H$465,C$3)</f>
@@ -6202,7 +6220,7 @@
       </c>
       <c r="D8" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A8,Master!$H$2:$H$465,D$3)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A8,Master!$H$2:$H$465,E$3)</f>
@@ -6284,7 +6302,7 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">SUM(B4:B10)</f>
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">SUM(C4:C10)</f>
@@ -6292,7 +6310,7 @@
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">SUM(D4:D10)</f>
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">SUM(E4:E10)</f>
@@ -6368,7 +6386,7 @@
       </c>
       <c r="B16" s="3" t="n">
         <f aca="false">COUNTIF(Master!$K$2:$K$465,A16)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -6398,7 +6416,7 @@
       </c>
       <c r="B18" s="3" t="n">
         <f aca="false">COUNTIF(Master!$K$2:$K$465,A18)</f>
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -6413,7 +6431,7 @@
       </c>
       <c r="B19" s="3" t="n">
         <f aca="false">COUNTIF(Master!$G$2:$G$465,"Read fully")</f>
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -6428,7 +6446,7 @@
       </c>
       <c r="B20" s="3" t="n">
         <f aca="false">COUNTIF(Master!$G$2:$G$465,"Not read")</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -6456,22 +6474,22 @@
   <dimension ref="A1:Q43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="3" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>26</v>
       </c>
@@ -6526,7 +6544,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>30</v>
       </c>
@@ -6591,7 +6609,7 @@
         <v>0.275</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>31</v>
       </c>
@@ -6656,7 +6674,7 @@
         <v>0.605263157894737</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>32</v>
       </c>
@@ -6666,7 +6684,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,D$18:D$42)</f>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,E$18:E$42)</f>
@@ -6674,7 +6692,7 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,F$18:F$42)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,G$18:G$42)</f>
@@ -6686,7 +6704,7 @@
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,I$18:I$42)</f>
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,J$18:J$42)</f>
@@ -6702,11 +6720,11 @@
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,M$18:M$42)</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,N$18:N$42)</f>
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,O$18:O$42)</f>
@@ -6714,14 +6732,14 @@
       </c>
       <c r="O7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,P$18:P$42)</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="P7" s="10" t="n">
         <f aca="false">IF(B7=0,0,1-L7/B7)</f>
-        <v>0.822429906542056</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.841121495327103</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
         <v>33</v>
       </c>
@@ -6786,7 +6804,7 @@
         <v>0.636363636363636</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>34</v>
       </c>
@@ -6851,7 +6869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>35</v>
       </c>
@@ -6916,7 +6934,7 @@
         <v>0.0512820512820513</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>36</v>
       </c>
@@ -6981,7 +6999,7 @@
         <v>0.111111111111111</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>7</v>
       </c>
@@ -6991,7 +7009,7 @@
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">SUM(C5:C11)</f>
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">SUM(D5:D11)</f>
@@ -6999,7 +7017,7 @@
       </c>
       <c r="E12" s="11" t="n">
         <f aca="false">SUM(E5:E11)</f>
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F12" s="11" t="n">
         <f aca="false">SUM(F5:F11)</f>
@@ -7011,7 +7029,7 @@
       </c>
       <c r="H12" s="11" t="n">
         <f aca="false">SUM(H5:H11)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I12" s="11" t="n">
         <f aca="false">SUM(I5:I11)</f>
@@ -7027,11 +7045,11 @@
       </c>
       <c r="L12" s="11" t="n">
         <f aca="false">SUM(L5:L11)</f>
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="M12" s="11" t="n">
         <f aca="false">SUM(M5:M11)</f>
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="N12" s="11" t="n">
         <f aca="false">SUM(N5:N11)</f>
@@ -7039,23 +7057,23 @@
       </c>
       <c r="O12" s="11" t="n">
         <f aca="false">SUM(O5:O11)</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="P12" s="12" t="n">
         <f aca="false">IF(B12=0,0,1-L12/B12)</f>
-        <v>0.353448275862069</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+        <v>0.357758620689655</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <f aca="false">COUNTA(Master!$D$2:$D$2000)-B12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>38</v>
       </c>
@@ -7113,7 +7131,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
         <v>41</v>
       </c>
@@ -7181,7 +7199,7 @@
         <v>0.275</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>42</v>
       </c>
@@ -7249,7 +7267,7 @@
         <v>0.605263157894737</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
         <v>43</v>
       </c>
@@ -7262,7 +7280,7 @@
       </c>
       <c r="D20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,D$17)</f>
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,E$17)</f>
@@ -7270,7 +7288,7 @@
       </c>
       <c r="F20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,F$17)</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,G$17)</f>
@@ -7282,7 +7300,7 @@
       </c>
       <c r="I20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$K$2:$K$2000,I$17)</f>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$K$2:$K$2000,J$17)</f>
@@ -7298,11 +7316,11 @@
       </c>
       <c r="M20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$K$2:$K$2000,M$17)</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$G$2:$G$2000,N$17)</f>
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$G$2:$G$2000,O$17)</f>
@@ -7310,14 +7328,14 @@
       </c>
       <c r="P20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$G$2:$G$2000,P$17)</f>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q20" s="10" t="n">
         <f aca="false">IF(C20=0,0,1-M20/C20)</f>
-        <v>0.870967741935484</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.89247311827957</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
         <v>44</v>
       </c>
@@ -7385,7 +7403,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
         <v>45</v>
       </c>
@@ -7453,7 +7471,7 @@
         <v>0.636363636363636</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
         <v>46</v>
       </c>
@@ -7521,7 +7539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
         <v>47</v>
       </c>
@@ -7589,7 +7607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
         <v>48</v>
       </c>
@@ -7657,7 +7675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
         <v>49</v>
       </c>
@@ -7725,7 +7743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
         <v>50</v>
       </c>
@@ -7793,7 +7811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
         <v>51</v>
       </c>
@@ -7861,7 +7879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
         <v>52</v>
       </c>
@@ -7929,7 +7947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
         <v>53</v>
       </c>
@@ -7997,7 +8015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
         <v>54</v>
       </c>
@@ -8065,7 +8083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
         <v>55</v>
       </c>
@@ -8133,7 +8151,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
         <v>56</v>
       </c>
@@ -8201,7 +8219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
         <v>57</v>
       </c>
@@ -8269,7 +8287,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
         <v>58</v>
       </c>
@@ -8337,7 +8355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
         <v>59</v>
       </c>
@@ -8405,7 +8423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
         <v>60</v>
       </c>
@@ -8473,7 +8491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
         <v>61</v>
       </c>
@@ -8541,7 +8559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
         <v>62</v>
       </c>
@@ -8609,7 +8627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
         <v>63</v>
       </c>
@@ -8677,7 +8695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
         <v>64</v>
       </c>
@@ -8745,7 +8763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
         <v>65</v>
       </c>
@@ -8813,7 +8831,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
         <v>7</v>
       </c>
@@ -8824,7 +8842,7 @@
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">SUM(D18:D42)</f>
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E43" s="11" t="n">
         <f aca="false">SUM(E18:E42)</f>
@@ -8832,7 +8850,7 @@
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">SUM(F18:F42)</f>
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G43" s="11" t="n">
         <f aca="false">SUM(G18:G42)</f>
@@ -8844,7 +8862,7 @@
       </c>
       <c r="I43" s="11" t="n">
         <f aca="false">SUM(I18:I42)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="J43" s="11" t="n">
         <f aca="false">SUM(J18:J42)</f>
@@ -8860,11 +8878,11 @@
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">SUM(M18:M42)</f>
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="N43" s="11" t="n">
         <f aca="false">SUM(N18:N42)</f>
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="O43" s="11" t="n">
         <f aca="false">SUM(O18:O42)</f>
@@ -8872,11 +8890,11 @@
       </c>
       <c r="P43" s="11" t="n">
         <f aca="false">SUM(P18:P42)</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="Q43" s="12" t="n">
         <f aca="false">IF(C43=0,0,1-M43/C43)</f>
-        <v>0.353448275862069</v>
+        <v>0.357758620689655</v>
       </c>
     </row>
   </sheetData>
@@ -25468,23 +25486,31 @@
       </c>
       <c r="F460" s="3"/>
       <c r="G460" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H460" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I460" s="3"/>
-      <c r="J460" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I460" s="3" t="s">
+        <v>1804</v>
+      </c>
+      <c r="J460" s="3" t="s">
+        <v>1805</v>
+      </c>
       <c r="K460" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L460" s="3"/>
-      <c r="M460" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="L460" s="3" t="s">
+        <v>1806</v>
+      </c>
+      <c r="M460" s="15" t="n">
+        <v>46327</v>
+      </c>
       <c r="N460" s="3"/>
     </row>
     <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A461" s="3" t="s">
-        <v>1804</v>
+        <v>1807</v>
       </c>
       <c r="B461" s="3" t="s">
         <v>80</v>
@@ -25493,10 +25519,10 @@
         <v>11</v>
       </c>
       <c r="D461" s="3" t="s">
-        <v>1805</v>
+        <v>1808</v>
       </c>
       <c r="E461" s="3" t="s">
-        <v>1806</v>
+        <v>1809</v>
       </c>
       <c r="F461" s="3"/>
       <c r="G461" s="3" t="s">
@@ -25516,7 +25542,7 @@
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A462" s="3" t="s">
-        <v>1807</v>
+        <v>1810</v>
       </c>
       <c r="B462" s="3" t="s">
         <v>80</v>
@@ -25525,13 +25551,13 @@
         <v>10</v>
       </c>
       <c r="D462" s="3" t="s">
-        <v>1808</v>
+        <v>1811</v>
       </c>
       <c r="E462" s="3" t="s">
-        <v>1809</v>
+        <v>1812</v>
       </c>
       <c r="F462" s="3" t="s">
-        <v>1810</v>
+        <v>1813</v>
       </c>
       <c r="G462" s="3" t="s">
         <v>22</v>
@@ -25540,25 +25566,25 @@
         <v>2</v>
       </c>
       <c r="I462" s="3" t="s">
-        <v>1811</v>
+        <v>1814</v>
       </c>
       <c r="J462" s="3"/>
       <c r="K462" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L462" s="3" t="s">
-        <v>1812</v>
+        <v>1815</v>
       </c>
       <c r="M462" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N462" s="3" t="s">
-        <v>1813</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A463" s="3" t="s">
-        <v>1814</v>
+        <v>1817</v>
       </c>
       <c r="B463" s="3" t="s">
         <v>80</v>
@@ -25567,13 +25593,13 @@
         <v>10</v>
       </c>
       <c r="D463" s="3" t="s">
-        <v>1815</v>
+        <v>1818</v>
       </c>
       <c r="E463" s="3" t="s">
-        <v>1816</v>
+        <v>1819</v>
       </c>
       <c r="F463" s="3" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="G463" s="3" t="s">
         <v>22</v>
@@ -25582,27 +25608,27 @@
         <v>3</v>
       </c>
       <c r="I463" s="3" t="s">
-        <v>1818</v>
+        <v>1821</v>
       </c>
       <c r="J463" s="3" t="s">
-        <v>1819</v>
+        <v>1822</v>
       </c>
       <c r="K463" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L463" s="3" t="s">
-        <v>1820</v>
+        <v>1823</v>
       </c>
       <c r="M463" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N463" s="3" t="s">
-        <v>1821</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A464" s="3" t="s">
-        <v>1822</v>
+        <v>1825</v>
       </c>
       <c r="B464" s="3" t="s">
         <v>80</v>
@@ -25611,30 +25637,38 @@
         <v>12</v>
       </c>
       <c r="D464" s="3" t="s">
-        <v>1823</v>
+        <v>1826</v>
       </c>
       <c r="E464" s="3" t="s">
-        <v>1824</v>
+        <v>1827</v>
       </c>
       <c r="F464" s="3"/>
       <c r="G464" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H464" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I464" s="3"/>
-      <c r="J464" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="I464" s="3" t="s">
+        <v>1828</v>
+      </c>
+      <c r="J464" s="3" t="s">
+        <v>1829</v>
+      </c>
       <c r="K464" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L464" s="3"/>
-      <c r="M464" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="L464" s="3" t="s">
+        <v>1830</v>
+      </c>
+      <c r="M464" s="15" t="n">
+        <v>46327</v>
+      </c>
       <c r="N464" s="3"/>
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A465" s="3" t="s">
-        <v>1825</v>
+        <v>1831</v>
       </c>
       <c r="B465" s="3" t="s">
         <v>80</v>
@@ -25643,10 +25677,10 @@
         <v>14</v>
       </c>
       <c r="D465" s="3" t="s">
-        <v>1826</v>
+        <v>1832</v>
       </c>
       <c r="E465" s="3" t="s">
-        <v>1827</v>
+        <v>1833</v>
       </c>
       <c r="F465" s="3"/>
       <c r="G465" s="3" t="s">
@@ -25661,7 +25695,7 @@
         <v>21</v>
       </c>
       <c r="L465" s="3" t="s">
-        <v>1828</v>
+        <v>1834</v>
       </c>
       <c r="M465" s="3"/>
       <c r="N465" s="3"/>

</xml_diff>

<commit_message>
LLM book rewritten in bullet style: Ch1-3 with interview corner, Ch4 glossary expanded to 140 entries; master updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ng7QdLy2CWEArt9UMzAUBr
</commit_message>
<xml_diff>
--- a/master/master.xlsx
+++ b/master/master.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5259" uniqueCount="2027">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5260" uniqueCount="2027">
   <si>
     <t xml:space="preserve">Master summary (live formulas)</t>
   </si>
@@ -1227,16 +1227,13 @@
     <t xml:space="preserve">38-term glossary with first-taught links</t>
   </si>
   <si>
-    <t xml:space="preserve">LLM › Ch 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terms for LangChain and MCP chapters not yet written (about 25 of its 38 terms)</t>
+    <t xml:space="preserve">LLM › Ch 4 (all its terms)</t>
   </si>
   <si>
     <t xml:space="preserve">Same terms as the transcription glossary, handled in one pass</t>
   </si>
   <si>
-    <t xml:space="preserve">Terms are added when their book chapters exist</t>
+    <t xml:space="preserve">All terms now in the rewritten glossary with chapter links.</t>
   </si>
   <si>
     <t xml:space="preserve">LC090</t>
@@ -1254,7 +1251,7 @@
     <t xml:space="preserve">Key table, .env workflow and git fixes were not in the books; Python, UV and VS Code link to Python Ch 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Not run: commands and URLs copied from the file; I did not open the URLs</t>
+    <t xml:space="preserve">Not run: commands and URLs copied from the file; I did not open the URLs | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC091</t>
@@ -1269,7 +1266,7 @@
     <t xml:space="preserve">Added five-phase arc, recurring projects and tooling</t>
   </si>
   <si>
-    <t xml:space="preserve">Class index table left out as navigation. README says classes 00 to 18; the transcript folder goes to class 23</t>
+    <t xml:space="preserve">Class index table left out as navigation. README says classes 00 to 18; the transcript folder goes to class 23 | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC092</t>
@@ -1659,7 +1656,7 @@
     <t xml:space="preserve">Added customs-form analogy, Google analogy, token example, 6x output price, controlled buffet vs a la carte, agent prompt with tools and tool-call flow</t>
   </si>
   <si>
-    <t xml:space="preserve">Whiteboard PDF: viewed the page. Price card ($5/$30, labelled 5.5) has no unit; check current prices. One student question has no answer on the slide</t>
+    <t xml:space="preserve">Whiteboard PDF: viewed the page. Price card ($5/$30, labelled 5.5) has no unit; check current prices. One student question has no answer on the slide | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC117</t>
@@ -1974,7 +1971,7 @@
     <t xml:space="preserve">Your choice: short original summary, no statistics or company claims</t>
   </si>
   <si>
-    <t xml:space="preserve">Marked 'Not for redistribution'; third-party marketing figures not verified</t>
+    <t xml:space="preserve">Marked 'Not for redistribution'; third-party marketing figures not verified | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC137</t>
@@ -2019,6 +2016,9 @@
     <t xml:space="preserve">Added the seven-file table and the no-offline-fallback note</t>
   </si>
   <si>
+    <t xml:space="preserve">LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
+  </si>
+  <si>
     <t xml:space="preserve">LC140</t>
   </si>
   <si>
@@ -2097,7 +2097,7 @@
     <t xml:space="preserve">Manual pipeline in Python Ch 3 › 3.6; get_weather is shown in LLM Ch 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Not run (needs keys)</t>
+    <t xml:space="preserve">Not run (needs keys) | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC144</t>
@@ -2118,7 +2118,7 @@
     <t xml:space="preserve">Added full schema, real replies and the three-calls example</t>
   </si>
   <si>
-    <t xml:space="preserve">Source quirks recorded: get_weather_schema mis-nested (parameters outside function); the three get_capital calls include two wrong arguments. Not run against a real model</t>
+    <t xml:space="preserve">Source quirks recorded: get_weather_schema mis-nested (parameters outside function); the three get_capital calls include two wrong arguments. Not run against a real model | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC145</t>
@@ -2139,7 +2139,7 @@
     <t xml:space="preserve">Added the terminal chat and the memory list</t>
   </si>
   <si>
-    <t xml:space="preserve">Run with a fake model: crashes with NameError on the first tool call (stray line with unquoted function); get_currency defined twice, second is pass and not in TOOL_SCHEMAS; scratch leftovers</t>
+    <t xml:space="preserve">Run with a fake model: crashes with NameError on the first tool call (stray line with unquoted function); get_currency defined twice, second is pass and not in TOOL_SCHEMAS; scratch leftovers | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC146</t>
@@ -2160,7 +2160,7 @@
     <t xml:space="preserve">Added three tools, calculator guard and session_state memory</t>
   </si>
   <si>
-    <t xml:space="preserve">Loop and calculator run with a fake model; currency API and Streamlit page not run</t>
+    <t xml:space="preserve">Loop and calculator run with a fake model; currency API and Streamlit page not run | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC147</t>
@@ -2181,7 +2181,7 @@
     <t xml:space="preserve">Not in the books before</t>
   </si>
   <si>
-    <t xml:space="preserve">JSON sample data, 44 lines</t>
+    <t xml:space="preserve">JSON sample data, 44 lines | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC148</t>
@@ -2268,7 +2268,7 @@
     <t xml:space="preserve">Added provider credits, tool-name clarity, decision fork, push-blocked note</t>
   </si>
   <si>
-    <t xml:space="preserve">Whiteboard PDF: read text and viewed the page. Placed the GitHub screenshot in Langchain Ch 1, not LLM Ch 2 as planned, because it concerns keys. Section number changed when Ch 1 was rewritten on 2026-11-01 (was 1.5)</t>
+    <t xml:space="preserve">Whiteboard PDF: read text and viewed the page. Placed the GitHub screenshot in Langchain Ch 1, not LLM Ch 2 as planned, because it concerns keys. Section number changed when Ch 1 was rewritten on 2026-11-01 (was 1.5) | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC155</t>
@@ -5235,7 +5235,7 @@
     <t xml:space="preserve">LLM book chapter 1 was empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Left out as logistics</t>
+    <t xml:space="preserve">Left out as logistics | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC419</t>
@@ -5292,7 +5292,7 @@
     <t xml:space="preserve">Pydantic › Ch 1 to 5; LLM › Ch 3 › 3.1</t>
   </si>
   <si>
-    <t xml:space="preserve">AI vocabulary placed in LLM book on your instruction; Pydantic snippets run and checked</t>
+    <t xml:space="preserve">AI vocabulary placed in LLM book on your instruction; Pydantic snippets run and checked | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC422</t>
@@ -5331,7 +5331,7 @@
     <t xml:space="preserve">LLM Ch 2 was empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Code excerpts copied from the summary; loop behaviour checked with a fake model</t>
+    <t xml:space="preserve">Code excerpts copied from the summary; loop behaviour checked with a fake model | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC424</t>
@@ -5604,7 +5604,7 @@
     <t xml:space="preserve">Added 2.0 vs 3.0 table, philosophy, hands-on flow, AgentOps, A2A</t>
   </si>
   <si>
-    <t xml:space="preserve">Demos, platform rules and schedule are logistics or marketing; say if you want the demos described</t>
+    <t xml:space="preserve">Demos, platform rules and schedule are logistics or marketing; say if you want the demos described | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC438</t>
@@ -5667,7 +5667,7 @@
     <t xml:space="preserve">Added typing background, comparison table, coercion table, EmailStr/HttpUrl/SecretStr, model_validator and order, inheritance Q&amp;A, AI term analogies</t>
   </si>
   <si>
-    <t xml:space="preserve">Course news and job reminder left out as no teaching content</t>
+    <t xml:space="preserve">Course news and job reminder left out as no teaching content | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC441</t>
@@ -5685,7 +5685,7 @@
     <t xml:space="preserve">Added memory and tools build-up, intern analogy, OpenRouter, Q&amp;A</t>
   </si>
   <si>
-    <t xml:space="preserve">Recap and song aside left out as no teaching content</t>
+    <t xml:space="preserve">Recap and song aside left out as no teaching content | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC442</t>
@@ -5706,7 +5706,7 @@
     <t xml:space="preserve">Added roles, knowledge cutoff, response shape and usage, max_tokens, structured-output ways, Q&amp;A</t>
   </si>
   <si>
-    <t xml:space="preserve">Class 02/03 'max_iterations' is called max_turns in the code files</t>
+    <t xml:space="preserve">Class 02/03 'max_iterations' is called max_turns in the code files | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC443</t>
@@ -6051,7 +6051,7 @@
     <t xml:space="preserve">Added further-reading links</t>
   </si>
   <si>
-    <t xml:space="preserve">Recording steps and student project showcase left out as logistics; links not opened</t>
+    <t xml:space="preserve">Recording steps and student project showcase left out as logistics; links not opened | LLM book rewritten in bullet style with interview corner, 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC462</t>
@@ -6066,16 +6066,16 @@
     <t xml:space="preserve">141-term glossary of the course</t>
   </si>
   <si>
-    <t xml:space="preserve">LLM › Ch 4 (28 entries)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Over 100 terms for LangChain and MCP chapters not yet written; also agentic loop, knowledge cutoff, max_tokens, messages, tool schema, vibe coding, harness</t>
+    <t xml:space="preserve">LLM › Ch 4 (140 entries)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only "vibe coding" has no teaching chapter (listed without a link)</t>
   </si>
   <si>
     <t xml:space="preserve">LLM glossary chapter was empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Glossary and its links come from a different repo (jakhmoladp/KrishNaik_acadmey_agentic_ai_3_0); I did not reuse those links</t>
+    <t xml:space="preserve">Definitions reworded; links point to this repo, not the source repo. Rewritten 2026-11-02.</t>
   </si>
   <si>
     <t xml:space="preserve">LC463</t>
@@ -6728,11 +6728,11 @@
       </c>
       <c r="B6" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A6,Master!$H$2:$H$465,B$3)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A6,Master!$H$2:$H$465,C$3)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3" t="n">
         <f aca="false">COUNTIFS(Master!$C$2:$C$465,$A6,Master!$H$2:$H$465,D$3)</f>
@@ -6878,11 +6878,11 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">SUM(B4:B10)</f>
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">SUM(C4:C10)</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">SUM(D4:D10)</f>
@@ -7260,11 +7260,11 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,D$18:D$42)</f>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,E$18:E$42)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUMIF($B$18:$B$42,$A7,F$18:F$42)</f>
@@ -7585,11 +7585,11 @@
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">SUM(C5:C11)</f>
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">SUM(D5:D11)</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="11" t="n">
         <f aca="false">SUM(E5:E11)</f>
@@ -7856,11 +7856,11 @@
       </c>
       <c r="D20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,D$17)</f>
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,E$17)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F20" s="9" t="n">
         <f aca="false">COUNTIFS(Master!$D$2:$D$2000,"*"&amp;$A20,Master!$H$2:$H$2000,F$17)</f>
@@ -9418,11 +9418,11 @@
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">SUM(D18:D42)</f>
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E43" s="11" t="n">
         <f aca="false">SUM(E18:E42)</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">SUM(F18:F42)</f>
@@ -12849,30 +12849,28 @@
         <v>22</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I90" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="J90" s="3" t="s">
-        <v>401</v>
-      </c>
+      <c r="J90" s="3"/>
       <c r="K90" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L90" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="M90" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="N90" s="3" t="s">
         <v>402</v>
-      </c>
-      <c r="M90" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="N90" s="3" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>80</v>
@@ -12881,13 +12879,13 @@
         <v>10</v>
       </c>
       <c r="D91" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="F91" s="3" t="s">
         <v>405</v>
-      </c>
-      <c r="E91" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="F91" s="3" t="s">
-        <v>406</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>22</v>
@@ -12896,25 +12894,25 @@
         <v>2</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="J91" s="3"/>
       <c r="K91" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L91" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="M91" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N91" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>80</v>
@@ -12929,7 +12927,7 @@
         <v>101</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>22</v>
@@ -12938,25 +12936,25 @@
         <v>2</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="J92" s="3"/>
       <c r="K92" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="M92" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N92" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>80</v>
@@ -12968,10 +12966,10 @@
         <v>101</v>
       </c>
       <c r="E93" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F93" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="F93" s="3" t="s">
-        <v>417</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>22</v>
@@ -12985,7 +12983,7 @@
         <v>17</v>
       </c>
       <c r="L93" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="M93" s="3" t="s">
         <v>92</v>
@@ -12994,7 +12992,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>80</v>
@@ -13003,13 +13001,13 @@
         <v>8</v>
       </c>
       <c r="D94" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="E94" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="E94" s="3" t="s">
+      <c r="F94" s="3" t="s">
         <v>421</v>
-      </c>
-      <c r="F94" s="3" t="s">
-        <v>422</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>22</v>
@@ -13018,25 +13016,25 @@
         <v>2</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J94" s="3"/>
       <c r="K94" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L94" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="M94" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N94" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>80</v>
@@ -13045,13 +13043,13 @@
         <v>8</v>
       </c>
       <c r="D95" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="E95" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="E95" s="3" t="s">
+      <c r="F95" s="3" t="s">
         <v>428</v>
-      </c>
-      <c r="F95" s="3" t="s">
-        <v>429</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>22</v>
@@ -13060,27 +13058,27 @@
         <v>3</v>
       </c>
       <c r="I95" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="J95" s="3" t="s">
         <v>430</v>
-      </c>
-      <c r="J95" s="3" t="s">
-        <v>431</v>
       </c>
       <c r="K95" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L95" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="M95" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N95" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>80</v>
@@ -13089,13 +13087,13 @@
         <v>8</v>
       </c>
       <c r="D96" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="E96" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="E96" s="3" t="s">
+      <c r="F96" s="3" t="s">
         <v>436</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>437</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>22</v>
@@ -13104,25 +13102,25 @@
         <v>2</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="J96" s="3"/>
       <c r="K96" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L96" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="M96" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N96" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>80</v>
@@ -13134,10 +13132,10 @@
         <v>101</v>
       </c>
       <c r="E97" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="F97" s="3" t="s">
-        <v>443</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>22</v>
@@ -13146,25 +13144,25 @@
         <v>2</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="J97" s="3"/>
       <c r="K97" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L97" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="M97" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N97" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>80</v>
@@ -13173,13 +13171,13 @@
         <v>8</v>
       </c>
       <c r="D98" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="E98" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="E98" s="3" t="s">
+      <c r="F98" s="3" t="s">
         <v>449</v>
-      </c>
-      <c r="F98" s="3" t="s">
-        <v>450</v>
       </c>
       <c r="G98" s="3" t="s">
         <v>22</v>
@@ -13188,25 +13186,25 @@
         <v>2</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="J98" s="3"/>
       <c r="K98" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L98" s="3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="M98" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N98" s="3" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>80</v>
@@ -13215,13 +13213,13 @@
         <v>8</v>
       </c>
       <c r="D99" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="E99" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="E99" s="3" t="s">
+      <c r="F99" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="F99" s="3" t="s">
-        <v>457</v>
       </c>
       <c r="G99" s="3" t="s">
         <v>22</v>
@@ -13230,14 +13228,14 @@
         <v>2</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="J99" s="3"/>
       <c r="K99" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M99" s="3" t="s">
         <v>92</v>
@@ -13246,7 +13244,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>80</v>
@@ -13258,7 +13256,7 @@
         <v>53</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="3" t="s">
@@ -13280,7 +13278,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>80</v>
@@ -13292,10 +13290,10 @@
         <v>101</v>
       </c>
       <c r="E101" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="F101" s="3" t="s">
         <v>463</v>
-      </c>
-      <c r="F101" s="3" t="s">
-        <v>464</v>
       </c>
       <c r="G101" s="3" t="s">
         <v>22</v>
@@ -13304,14 +13302,14 @@
         <v>2</v>
       </c>
       <c r="I101" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J101" s="3"/>
       <c r="K101" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="M101" s="3" t="s">
         <v>92</v>
@@ -13320,7 +13318,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>80</v>
@@ -13332,10 +13330,10 @@
         <v>205</v>
       </c>
       <c r="E102" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="F102" s="3" t="s">
         <v>467</v>
-      </c>
-      <c r="F102" s="3" t="s">
-        <v>468</v>
       </c>
       <c r="G102" s="3" t="s">
         <v>22</v>
@@ -13344,14 +13342,14 @@
         <v>2</v>
       </c>
       <c r="I102" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J102" s="3"/>
       <c r="K102" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L102" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="M102" s="3" t="s">
         <v>92</v>
@@ -13360,7 +13358,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>80</v>
@@ -13372,7 +13370,7 @@
         <v>130</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3" t="s">
@@ -13394,7 +13392,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B104" s="3" t="s">
         <v>80</v>
@@ -13403,10 +13401,10 @@
         <v>8</v>
       </c>
       <c r="D104" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="E104" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="E104" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="F104" s="3"/>
       <c r="G104" s="3" t="s">
@@ -13421,14 +13419,14 @@
         <v>21</v>
       </c>
       <c r="L104" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M104" s="3"/>
       <c r="N104" s="3"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B105" s="3" t="s">
         <v>80</v>
@@ -13440,7 +13438,7 @@
         <v>148</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="3" t="s">
@@ -13462,7 +13460,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>80</v>
@@ -13471,13 +13469,13 @@
         <v>8</v>
       </c>
       <c r="D106" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E106" s="3" t="s">
         <v>479</v>
       </c>
-      <c r="E106" s="3" t="s">
+      <c r="F106" s="3" t="s">
         <v>480</v>
-      </c>
-      <c r="F106" s="3" t="s">
-        <v>481</v>
       </c>
       <c r="G106" s="3" t="s">
         <v>22</v>
@@ -13486,25 +13484,25 @@
         <v>2</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="J106" s="3"/>
       <c r="K106" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L106" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="M106" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N106" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>80</v>
@@ -13513,13 +13511,13 @@
         <v>8</v>
       </c>
       <c r="D107" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="E107" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="E107" s="3" t="s">
+      <c r="F107" s="3" t="s">
         <v>486</v>
-      </c>
-      <c r="F107" s="3" t="s">
-        <v>487</v>
       </c>
       <c r="G107" s="3" t="s">
         <v>22</v>
@@ -13528,25 +13526,25 @@
         <v>2</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="J107" s="3"/>
       <c r="K107" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L107" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M107" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N107" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>80</v>
@@ -13555,13 +13553,13 @@
         <v>8</v>
       </c>
       <c r="D108" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="E108" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="E108" s="3" t="s">
+      <c r="F108" s="3" t="s">
         <v>492</v>
-      </c>
-      <c r="F108" s="3" t="s">
-        <v>493</v>
       </c>
       <c r="G108" s="3" t="s">
         <v>22</v>
@@ -13570,25 +13568,25 @@
         <v>2</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="J108" s="3"/>
       <c r="K108" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L108" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="M108" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N108" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>80</v>
@@ -13600,7 +13598,7 @@
         <v>53</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="F109" s="3"/>
       <c r="G109" s="3" t="s">
@@ -13622,7 +13620,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>80</v>
@@ -13631,13 +13629,13 @@
         <v>9</v>
       </c>
       <c r="D110" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="E110" s="3" t="s">
         <v>500</v>
       </c>
-      <c r="E110" s="3" t="s">
+      <c r="F110" s="3" t="s">
         <v>501</v>
-      </c>
-      <c r="F110" s="3" t="s">
-        <v>502</v>
       </c>
       <c r="G110" s="3" t="s">
         <v>22</v>
@@ -13646,25 +13644,25 @@
         <v>2</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="J110" s="3"/>
       <c r="K110" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L110" s="3" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="M110" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N110" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>80</v>
@@ -13673,13 +13671,13 @@
         <v>9</v>
       </c>
       <c r="D111" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="E111" s="3" t="s">
         <v>507</v>
       </c>
-      <c r="E111" s="3" t="s">
+      <c r="F111" s="3" t="s">
         <v>508</v>
-      </c>
-      <c r="F111" s="3" t="s">
-        <v>509</v>
       </c>
       <c r="G111" s="3" t="s">
         <v>22</v>
@@ -13688,27 +13686,27 @@
         <v>3</v>
       </c>
       <c r="I111" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="J111" s="3" t="s">
         <v>510</v>
-      </c>
-      <c r="J111" s="3" t="s">
-        <v>511</v>
       </c>
       <c r="K111" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="M111" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N111" s="3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>80</v>
@@ -13720,10 +13718,10 @@
         <v>101</v>
       </c>
       <c r="E112" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="F112" s="3" t="s">
         <v>515</v>
-      </c>
-      <c r="F112" s="3" t="s">
-        <v>516</v>
       </c>
       <c r="G112" s="3" t="s">
         <v>22</v>
@@ -13732,14 +13730,14 @@
         <v>2</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="J112" s="3"/>
       <c r="K112" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L112" s="3" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="M112" s="3" t="s">
         <v>92</v>
@@ -13748,7 +13746,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>80</v>
@@ -13760,10 +13758,10 @@
         <v>205</v>
       </c>
       <c r="E113" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="F113" s="3" t="s">
         <v>520</v>
-      </c>
-      <c r="F113" s="3" t="s">
-        <v>521</v>
       </c>
       <c r="G113" s="3" t="s">
         <v>22</v>
@@ -13777,18 +13775,18 @@
         <v>17</v>
       </c>
       <c r="L113" s="3" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="M113" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N113" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>80</v>
@@ -13800,7 +13798,7 @@
         <v>130</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="3" t="s">
@@ -13822,7 +13820,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>80</v>
@@ -13831,13 +13829,13 @@
         <v>9</v>
       </c>
       <c r="D115" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="E115" s="3" t="s">
         <v>527</v>
       </c>
-      <c r="E115" s="3" t="s">
+      <c r="F115" s="3" t="s">
         <v>528</v>
-      </c>
-      <c r="F115" s="3" t="s">
-        <v>529</v>
       </c>
       <c r="G115" s="3" t="s">
         <v>22</v>
@@ -13851,18 +13849,18 @@
         <v>17</v>
       </c>
       <c r="L115" s="3" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="M115" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N115" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>80</v>
@@ -13871,13 +13869,13 @@
         <v>8</v>
       </c>
       <c r="D116" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="E116" s="3" t="s">
         <v>532</v>
       </c>
-      <c r="E116" s="3" t="s">
+      <c r="F116" s="3" t="s">
         <v>533</v>
-      </c>
-      <c r="F116" s="3" t="s">
-        <v>534</v>
       </c>
       <c r="G116" s="3" t="s">
         <v>22</v>
@@ -13886,25 +13884,25 @@
         <v>2</v>
       </c>
       <c r="I116" s="3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="J116" s="3"/>
       <c r="K116" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L116" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="M116" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N116" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>80</v>
@@ -13913,13 +13911,13 @@
         <v>8</v>
       </c>
       <c r="D117" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="E117" s="3" t="s">
         <v>539</v>
       </c>
-      <c r="E117" s="3" t="s">
+      <c r="F117" s="3" t="s">
         <v>540</v>
-      </c>
-      <c r="F117" s="3" t="s">
-        <v>541</v>
       </c>
       <c r="G117" s="3" t="s">
         <v>22</v>
@@ -13928,25 +13926,25 @@
         <v>2</v>
       </c>
       <c r="I117" s="3" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="J117" s="3"/>
       <c r="K117" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L117" s="3" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="M117" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N117" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>80</v>
@@ -13955,13 +13953,13 @@
         <v>8</v>
       </c>
       <c r="D118" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E118" s="3" t="s">
         <v>546</v>
       </c>
-      <c r="E118" s="3" t="s">
+      <c r="F118" s="3" t="s">
         <v>547</v>
-      </c>
-      <c r="F118" s="3" t="s">
-        <v>548</v>
       </c>
       <c r="G118" s="3" t="s">
         <v>22</v>
@@ -13970,25 +13968,25 @@
         <v>2</v>
       </c>
       <c r="I118" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="J118" s="3"/>
       <c r="K118" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L118" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="M118" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N118" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>80</v>
@@ -14000,10 +13998,10 @@
         <v>101</v>
       </c>
       <c r="E119" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="F119" s="3" t="s">
         <v>553</v>
-      </c>
-      <c r="F119" s="3" t="s">
-        <v>554</v>
       </c>
       <c r="G119" s="3" t="s">
         <v>22</v>
@@ -14012,25 +14010,25 @@
         <v>2</v>
       </c>
       <c r="I119" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="J119" s="3"/>
       <c r="K119" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L119" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="M119" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N119" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>80</v>
@@ -14039,13 +14037,13 @@
         <v>8</v>
       </c>
       <c r="D120" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="E120" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="E120" s="3" t="s">
+      <c r="F120" s="3" t="s">
         <v>560</v>
-      </c>
-      <c r="F120" s="3" t="s">
-        <v>561</v>
       </c>
       <c r="G120" s="3" t="s">
         <v>22</v>
@@ -14054,25 +14052,25 @@
         <v>2</v>
       </c>
       <c r="I120" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="J120" s="3"/>
       <c r="K120" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L120" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="M120" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N120" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>80</v>
@@ -14081,13 +14079,13 @@
         <v>9</v>
       </c>
       <c r="D121" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="E121" s="3" t="s">
         <v>564</v>
       </c>
-      <c r="E121" s="3" t="s">
+      <c r="F121" s="3" t="s">
         <v>565</v>
-      </c>
-      <c r="F121" s="3" t="s">
-        <v>566</v>
       </c>
       <c r="G121" s="3" t="s">
         <v>22</v>
@@ -14096,25 +14094,25 @@
         <v>2</v>
       </c>
       <c r="I121" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J121" s="3"/>
       <c r="K121" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L121" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="M121" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N121" s="3" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>80</v>
@@ -14123,10 +14121,10 @@
         <v>8</v>
       </c>
       <c r="D122" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="E122" s="3" t="s">
         <v>571</v>
-      </c>
-      <c r="E122" s="3" t="s">
-        <v>572</v>
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="3" t="s">
@@ -14141,7 +14139,7 @@
         <v>21</v>
       </c>
       <c r="L122" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M122" s="3" t="s">
         <v>92</v>
@@ -14150,7 +14148,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>80</v>
@@ -14159,10 +14157,10 @@
         <v>8</v>
       </c>
       <c r="D123" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="E123" s="3" t="s">
         <v>575</v>
-      </c>
-      <c r="E123" s="3" t="s">
-        <v>576</v>
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="3" t="s">
@@ -14177,7 +14175,7 @@
         <v>21</v>
       </c>
       <c r="L123" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M123" s="3" t="s">
         <v>92</v>
@@ -14186,7 +14184,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>80</v>
@@ -14195,10 +14193,10 @@
         <v>8</v>
       </c>
       <c r="D124" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="E124" s="3" t="s">
         <v>578</v>
-      </c>
-      <c r="E124" s="3" t="s">
-        <v>579</v>
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="3" t="s">
@@ -14213,7 +14211,7 @@
         <v>21</v>
       </c>
       <c r="L124" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M124" s="3" t="s">
         <v>92</v>
@@ -14222,7 +14220,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>80</v>
@@ -14231,10 +14229,10 @@
         <v>8</v>
       </c>
       <c r="D125" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="E125" s="3" t="s">
         <v>581</v>
-      </c>
-      <c r="E125" s="3" t="s">
-        <v>582</v>
       </c>
       <c r="F125" s="3"/>
       <c r="G125" s="3" t="s">
@@ -14249,7 +14247,7 @@
         <v>21</v>
       </c>
       <c r="L125" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M125" s="3" t="s">
         <v>92</v>
@@ -14258,7 +14256,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>80</v>
@@ -14267,13 +14265,13 @@
         <v>8</v>
       </c>
       <c r="D126" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="E126" s="3" t="s">
         <v>584</v>
       </c>
-      <c r="E126" s="3" t="s">
+      <c r="F126" s="3" t="s">
         <v>585</v>
-      </c>
-      <c r="F126" s="3" t="s">
-        <v>586</v>
       </c>
       <c r="G126" s="3" t="s">
         <v>22</v>
@@ -14282,25 +14280,25 @@
         <v>2</v>
       </c>
       <c r="I126" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="J126" s="3"/>
       <c r="K126" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L126" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="M126" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N126" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>80</v>
@@ -14309,13 +14307,13 @@
         <v>8</v>
       </c>
       <c r="D127" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="E127" s="3" t="s">
         <v>589</v>
       </c>
-      <c r="E127" s="3" t="s">
+      <c r="F127" s="3" t="s">
         <v>590</v>
-      </c>
-      <c r="F127" s="3" t="s">
-        <v>591</v>
       </c>
       <c r="G127" s="3" t="s">
         <v>22</v>
@@ -14324,25 +14322,25 @@
         <v>2</v>
       </c>
       <c r="I127" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="J127" s="3"/>
       <c r="K127" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L127" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="M127" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N127" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>80</v>
@@ -14351,13 +14349,13 @@
         <v>8</v>
       </c>
       <c r="D128" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="E128" s="3" t="s">
         <v>595</v>
       </c>
-      <c r="E128" s="3" t="s">
+      <c r="F128" s="3" t="s">
         <v>596</v>
-      </c>
-      <c r="F128" s="3" t="s">
-        <v>597</v>
       </c>
       <c r="G128" s="3" t="s">
         <v>22</v>
@@ -14366,25 +14364,25 @@
         <v>2</v>
       </c>
       <c r="I128" s="3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="J128" s="3"/>
       <c r="K128" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L128" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M128" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N128" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>80</v>
@@ -14393,13 +14391,13 @@
         <v>8</v>
       </c>
       <c r="D129" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="E129" s="3" t="s">
         <v>601</v>
       </c>
-      <c r="E129" s="3" t="s">
+      <c r="F129" s="3" t="s">
         <v>602</v>
-      </c>
-      <c r="F129" s="3" t="s">
-        <v>603</v>
       </c>
       <c r="G129" s="3" t="s">
         <v>22</v>
@@ -14408,25 +14406,25 @@
         <v>2</v>
       </c>
       <c r="I129" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="J129" s="3"/>
       <c r="K129" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L129" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="M129" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N129" s="3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>80</v>
@@ -14435,13 +14433,13 @@
         <v>8</v>
       </c>
       <c r="D130" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="E130" s="3" t="s">
         <v>608</v>
       </c>
-      <c r="E130" s="3" t="s">
+      <c r="F130" s="3" t="s">
         <v>609</v>
-      </c>
-      <c r="F130" s="3" t="s">
-        <v>610</v>
       </c>
       <c r="G130" s="3" t="s">
         <v>22</v>
@@ -14450,25 +14448,25 @@
         <v>2</v>
       </c>
       <c r="I130" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="J130" s="3"/>
       <c r="K130" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L130" s="3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="M130" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N130" s="3" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B131" s="3" t="s">
         <v>80</v>
@@ -14477,13 +14475,13 @@
         <v>8</v>
       </c>
       <c r="D131" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="E131" s="3" t="s">
         <v>615</v>
       </c>
-      <c r="E131" s="3" t="s">
+      <c r="F131" s="3" t="s">
         <v>616</v>
-      </c>
-      <c r="F131" s="3" t="s">
-        <v>617</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>22</v>
@@ -14492,25 +14490,25 @@
         <v>2</v>
       </c>
       <c r="I131" s="3" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="J131" s="3"/>
       <c r="K131" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L131" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M131" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N131" s="3" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>80</v>
@@ -14519,13 +14517,13 @@
         <v>8</v>
       </c>
       <c r="D132" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="E132" s="3" t="s">
         <v>621</v>
       </c>
-      <c r="E132" s="3" t="s">
+      <c r="F132" s="3" t="s">
         <v>622</v>
-      </c>
-      <c r="F132" s="3" t="s">
-        <v>623</v>
       </c>
       <c r="G132" s="3" t="s">
         <v>22</v>
@@ -14534,25 +14532,25 @@
         <v>2</v>
       </c>
       <c r="I132" s="3" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="J132" s="3"/>
       <c r="K132" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L132" s="3" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="M132" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N132" s="3" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>80</v>
@@ -14561,13 +14559,13 @@
         <v>9</v>
       </c>
       <c r="D133" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="E133" s="3" t="s">
         <v>627</v>
       </c>
-      <c r="E133" s="3" t="s">
+      <c r="F133" s="3" t="s">
         <v>628</v>
-      </c>
-      <c r="F133" s="3" t="s">
-        <v>629</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>22</v>
@@ -14576,25 +14574,25 @@
         <v>2</v>
       </c>
       <c r="I133" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J133" s="3"/>
       <c r="K133" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L133" s="3" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="M133" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N133" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>80</v>
@@ -14603,13 +14601,13 @@
         <v>9</v>
       </c>
       <c r="D134" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="E134" s="3" t="s">
         <v>633</v>
       </c>
-      <c r="E134" s="3" t="s">
+      <c r="F134" s="3" t="s">
         <v>634</v>
-      </c>
-      <c r="F134" s="3" t="s">
-        <v>635</v>
       </c>
       <c r="G134" s="3" t="s">
         <v>22</v>
@@ -14618,25 +14616,25 @@
         <v>2</v>
       </c>
       <c r="I134" s="3" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J134" s="3"/>
       <c r="K134" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L134" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M134" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N134" s="3" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>80</v>
@@ -14648,7 +14646,7 @@
         <v>130</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F135" s="3"/>
       <c r="G135" s="3" t="s">
@@ -14670,7 +14668,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>80</v>
@@ -14682,7 +14680,7 @@
         <v>148</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F136" s="3"/>
       <c r="G136" s="3" t="s">
@@ -14704,7 +14702,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>80</v>
@@ -14713,13 +14711,13 @@
         <v>10</v>
       </c>
       <c r="D137" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="E137" s="3" t="s">
         <v>643</v>
       </c>
-      <c r="E137" s="3" t="s">
+      <c r="F137" s="3" t="s">
         <v>644</v>
-      </c>
-      <c r="F137" s="3" t="s">
-        <v>645</v>
       </c>
       <c r="G137" s="3" t="s">
         <v>22</v>
@@ -14728,27 +14726,27 @@
         <v>3</v>
       </c>
       <c r="I137" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="J137" s="3" t="s">
         <v>646</v>
-      </c>
-      <c r="J137" s="3" t="s">
-        <v>647</v>
       </c>
       <c r="K137" s="3" t="s">
         <v>19</v>
       </c>
       <c r="L137" s="3" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="M137" s="3" t="s">
         <v>109</v>
       </c>
       <c r="N137" s="3" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>80</v>
@@ -14760,10 +14758,10 @@
         <v>101</v>
       </c>
       <c r="E138" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="F138" s="3" t="s">
         <v>651</v>
-      </c>
-      <c r="F138" s="3" t="s">
-        <v>652</v>
       </c>
       <c r="G138" s="3" t="s">
         <v>22</v>
@@ -14773,24 +14771,24 @@
       </c>
       <c r="I138" s="3"/>
       <c r="J138" s="3" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="K138" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L138" s="3" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="M138" s="3" t="s">
         <v>92</v>
       </c>
       <c r="N138" s="3" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="3" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>80</v>
@@ -14802,7 +14800,7 @@
         <v>54</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F139" s="3"/>
       <c r="G139" s="3" t="s">
@@ -14821,12 +14819,12 @@
       </c>
       <c r="M139" s="3"/>
       <c r="N139" s="3" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>80</v>
@@ -14838,10 +14836,10 @@
         <v>101</v>
       </c>
       <c r="E140" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="F140" s="3" t="s">
         <v>660</v>
-      </c>
-      <c r="F140" s="3" t="s">
-        <v>661</v>
       </c>
       <c r="G140" s="3" t="s">
         <v>22</v>
@@ -14850,19 +14848,21 @@
         <v>2</v>
       </c>
       <c r="I140" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="J140" s="3"/>
       <c r="K140" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L140" s="3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="M140" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="N140" s="3"/>
+      <c r="N140" s="3" t="s">
+        <v>663</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="3" t="s">
@@ -15231,7 +15231,7 @@
       </c>
       <c r="M149" s="3"/>
       <c r="N149" s="3" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15272,7 +15272,9 @@
       <c r="M150" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="N150" s="3"/>
+      <c r="N150" s="3" t="s">
+        <v>663</v>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="3" t="s">
@@ -15323,7 +15325,7 @@
         <v>11</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E152" s="3" t="s">
         <v>731</v>
@@ -15789,7 +15791,7 @@
         <v>11</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E164" s="3" t="s">
         <v>788</v>
@@ -16263,7 +16265,7 @@
         <v>11</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E176" s="3" t="s">
         <v>841</v>
@@ -16281,7 +16283,7 @@
         <v>21</v>
       </c>
       <c r="L176" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M176" s="3"/>
       <c r="N176" s="3" t="s">
@@ -21223,7 +21225,7 @@
         <v>13</v>
       </c>
       <c r="D303" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E303" s="3" t="s">
         <v>1355</v>
@@ -21385,7 +21387,7 @@
         <v>21</v>
       </c>
       <c r="L307" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M307" s="3"/>
       <c r="N307" s="3"/>
@@ -21553,7 +21555,7 @@
         <v>13</v>
       </c>
       <c r="D312" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E312" s="3" t="s">
         <v>1388</v>
@@ -25187,7 +25189,7 @@
         <v>21</v>
       </c>
       <c r="L412" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M412" s="3"/>
       <c r="N412" s="3"/>
@@ -25203,7 +25205,7 @@
         <v>13</v>
       </c>
       <c r="D413" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E413" s="3" t="s">
         <v>1705</v>
@@ -25221,7 +25223,7 @@
         <v>21</v>
       </c>
       <c r="L413" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M413" s="3"/>
       <c r="N413" s="3"/>
@@ -27294,7 +27296,7 @@
         <v>2015</v>
       </c>
       <c r="M463" s="3" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="N463" s="3" t="s">
         <v>2016</v>

</xml_diff>